<commit_message>
Replace example split with the original split
</commit_message>
<xml_diff>
--- a/scan_split_example.xlsx
+++ b/scan_split_example.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/soupee/Documents/GitHub/NeuroBOLT-code/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/soupee/Desktop/neurips-eegfmri/GitHub/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D3D2632-4F1C-E34D-B555-EBC417FFC8A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C739AB6-AD94-724E-8B54-D6527BD93506}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2240" yWindow="1200" windowWidth="25760" windowHeight="15540" xr2:uid="{607F6B7C-1548-BE48-BA1D-728E01B417ED}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
   <si>
     <t>scan_name</t>
   </si>
@@ -54,9 +54,6 @@
     <t>sub02-scan01</t>
   </si>
   <si>
-    <t>sub03-scan01</t>
-  </si>
-  <si>
     <t>sub04-scan01</t>
   </si>
   <si>
@@ -70,6 +67,72 @@
   </si>
   <si>
     <t>sub07-scan02</t>
+  </si>
+  <si>
+    <t>sub03-scan02</t>
+  </si>
+  <si>
+    <t>sub08-scan01</t>
+  </si>
+  <si>
+    <t>sub08-scan02</t>
+  </si>
+  <si>
+    <t>sub09-scan01</t>
+  </si>
+  <si>
+    <t>sub09-scan02</t>
+  </si>
+  <si>
+    <t>sub10-scan02</t>
+  </si>
+  <si>
+    <t>sub11-scan01</t>
+  </si>
+  <si>
+    <t>sub12-scan01</t>
+  </si>
+  <si>
+    <t>sub12-scan02</t>
+  </si>
+  <si>
+    <t>sub13-scan01</t>
+  </si>
+  <si>
+    <t>sub13-scan02</t>
+  </si>
+  <si>
+    <t>sub14-scan01</t>
+  </si>
+  <si>
+    <t>sub14-scan02</t>
+  </si>
+  <si>
+    <t>sub15-scan01</t>
+  </si>
+  <si>
+    <t>sub16-scan01</t>
+  </si>
+  <si>
+    <t>sub17-scan02</t>
+  </si>
+  <si>
+    <t>sub18-scan01</t>
+  </si>
+  <si>
+    <t>sub19-scan02</t>
+  </si>
+  <si>
+    <t>sub20-scan01</t>
+  </si>
+  <si>
+    <t>sub20-scan02</t>
+  </si>
+  <si>
+    <t>sub21-scan01</t>
+  </si>
+  <si>
+    <t>sub22-scan01</t>
   </si>
 </sst>
 </file>
@@ -478,7 +541,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C4">
         <v>1</v>
@@ -490,7 +553,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C5">
         <v>1</v>
@@ -502,7 +565,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C6">
         <v>1</v>
@@ -514,7 +577,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D7">
         <v>1</v>
@@ -526,7 +589,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E8">
         <v>1</v>
@@ -538,75 +601,243 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E9">
+        <v>1</v>
+      </c>
+      <c r="F9" s="1"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>13</v>
+      </c>
+      <c r="C11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A12">
         <v>11</v>
       </c>
-      <c r="E9">
-        <v>1</v>
-      </c>
-      <c r="F9" s="1"/>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A10" s="1"/>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A11" s="1"/>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A12" s="1"/>
+      <c r="B12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C12">
+        <v>1</v>
+      </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A13" s="1"/>
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>15</v>
+      </c>
+      <c r="C13">
+        <v>1</v>
+      </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A14" s="1"/>
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>16</v>
+      </c>
+      <c r="C14">
+        <v>1</v>
+      </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A15" s="1"/>
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>17</v>
+      </c>
+      <c r="E15">
+        <v>1</v>
+      </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A16" s="1"/>
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>18</v>
+      </c>
+      <c r="C16">
+        <v>1</v>
+      </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A17" s="1"/>
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
+        <v>19</v>
+      </c>
+      <c r="C17">
+        <v>1</v>
+      </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A18" s="1"/>
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
+        <v>20</v>
+      </c>
+      <c r="D18">
+        <v>1</v>
+      </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A19" s="1"/>
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
+        <v>21</v>
+      </c>
+      <c r="D19">
+        <v>1</v>
+      </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A20" s="1"/>
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="s">
+        <v>22</v>
+      </c>
+      <c r="C20">
+        <v>1</v>
+      </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A21" s="1"/>
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="s">
+        <v>23</v>
+      </c>
+      <c r="C21">
+        <v>1</v>
+      </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A22" s="1"/>
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" t="s">
+        <v>24</v>
+      </c>
+      <c r="D22">
+        <v>1</v>
+      </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A23" s="1"/>
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" t="s">
+        <v>25</v>
+      </c>
+      <c r="E23">
+        <v>1</v>
+      </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A24" s="1"/>
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" t="s">
+        <v>26</v>
+      </c>
+      <c r="C24">
+        <v>1</v>
+      </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A25" s="1"/>
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" t="s">
+        <v>27</v>
+      </c>
+      <c r="E25">
+        <v>1</v>
+      </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A26" s="1"/>
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" t="s">
+        <v>28</v>
+      </c>
+      <c r="C26">
+        <v>1</v>
+      </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A27" s="1"/>
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" t="s">
+        <v>29</v>
+      </c>
+      <c r="C27">
+        <v>1</v>
+      </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A28" s="1"/>
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" t="s">
+        <v>30</v>
+      </c>
+      <c r="C28">
+        <v>1</v>
+      </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A29" s="1"/>
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29" t="s">
+        <v>31</v>
+      </c>
+      <c r="E29">
+        <v>1</v>
+      </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A30" s="1"/>
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30" t="s">
+        <v>32</v>
+      </c>
+      <c r="D30">
+        <v>1</v>
+      </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="F31" s="1"/>

</xml_diff>